<commit_message>
More GTFS Inputs - WIP at the moment, flow crashes!
</commit_message>
<xml_diff>
--- a/data/input/GTFS/depot_locations.xlsx
+++ b/data/input/GTFS/depot_locations.xlsx
@@ -1,16 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arbeit/Documents/Arbeit/Software/eflips-x/data/input/GTFS/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A6814FB-5112-3A49-9726-5CC7F1438094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="23500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -20,292 +25,463 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="92">
-  <si>
-    <t xml:space="preserve">file_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">agency_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">agency_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">coords</t>
-  </si>
-  <si>
-    <t xml:space="preserve">capacity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">address</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VBB.zip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S-Bahn Berlin GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N/A – pure rail operator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oberhavel Verkehrsgesellschaft mbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oranienburger Depot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">52.74557505576078, 13.192751192327316</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annahofer Str. 1A, 16515 Oranienburg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verkehrsbetriebe Brandenburg an der Havel GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betriebshof Hohenstücken</t>
-  </si>
-  <si>
-    <t xml:space="preserve">52.428767636612015, 12.533650229827478</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Upstallstraße 18, 14772 Brandenburg an der Havel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stadtverkehrsgesellschaft mbH Frankfurt (Oder)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betriebshof SVF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">52.32006508527503, 14.537452913933096</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Böttnerstraße 1, 15232 Frankfurt (Oder)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Havelbus Verkehrsgesellschaft mbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betriebshof Nauen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">52.61504442529055, 12.886949093497295</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ludwig-Jahn-Straße 1, 14641 Nauen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uckermärkische Verkehrsgesellschaft mbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uckermärkische Verkehrsgesellschaft</t>
-  </si>
-  <si>
-    <t xml:space="preserve">53.07084676329792, 14.261990922515063</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Steinstraße 5, 16303 Schwedt/Oder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DB Regio AG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Günter Anger Güterverkehrs GmbH &amp; Co. Omnibusvermietung KG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verkehrsbetrieb Potsdam GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ViP Betriebshof</t>
-  </si>
-  <si>
-    <t xml:space="preserve">52.37628875873694, 13.112412796506037</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fiktiver Betriebshof Sanssouci</t>
-  </si>
-  <si>
-    <t xml:space="preserve">52.40497313856915, 13.038360454025698</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Barnimer Busgesellschaft mbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betriebshof Nordend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">52.84967429943032, 13.814701141381143</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Poratzstraße 68, 16225 Eberswalde</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verkehrsgesellschaft Teltow-Fläming mbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betriebshof Luckenwalde</t>
-  </si>
-  <si>
-    <t xml:space="preserve">52.08339028518163, 13.160681509418481</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forststraße 16, 14943 Luckenwalde</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regionale Verkehrsgesellschaft Dahme-Spreewald mbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nissanstr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">51.859601652429475, 13.733812378374783</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nissanstraße 7, 15926 Luckau</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verkehrsmanagement Elbe-Elster GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verkehrsgesellschaft Oberspreewald-Lausitz mbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fritz Behrendt OHG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glaser</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Schöneicher Rüdersdorfer Straßenbahn GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strausberger Eisenbahn GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cottbusverkehr GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Walther-Rathenau-Straße</t>
-  </si>
-  <si>
-    <t xml:space="preserve">51.789058228725466, 14.332313340030659</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Walther-Rathenau-Straße 38, 03044 Cottbus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Busverkehr Oder-Spree GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">James-Watt-Str</t>
-  </si>
-  <si>
-    <t xml:space="preserve">52.35627786718695, 14.087576948727444</t>
-  </si>
-  <si>
-    <t xml:space="preserve">James-Watt-Straße 4, 15517 Fürstenwalde</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NEB Betriebsgesellschaft mbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A. Reich GmbH Busbetrieb</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sabinchen Touristik GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Busverkehr Gerd Schmidt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ORP Ostprignitz-Ruppiner Personennahverkehrsgesellschaft mbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perleberger Str</t>
-  </si>
-  <si>
-    <t xml:space="preserve">52.95172629551461, 12.379063105024942</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perleberger Str. 64, 16866 Kyritz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ODEG Ostdeutsche Eisenbahn GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hanseatische Eisenbahn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DB Regio Bus Ost GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lange</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Berliner Verkehrsbetriebe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prignitzbus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mobus Märkisch-Oderland Bus GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betriebshof Strausberg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">52.54829721100754, 13.860390543594225</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Märkische Straße 3, 15344 Strausberg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">regiobus Potsdam Mittelmark GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Am Betriebshof</t>
-  </si>
-  <si>
-    <t xml:space="preserve">52.14486495791746, 12.613296403587013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brücker Landstraße 22, 14806 Bad Belzig</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mitteldeutsche Regiobahn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betreiber: ecoVista</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SWU.zip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SWU Verkehr GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SWU Betriebshof</t>
-  </si>
-  <si>
-    <t xml:space="preserve">48.39658695394624, 9.967748831666805</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bauhoferstraße 9, 89077 Ulm</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="150">
+  <si>
+    <t>file_name</t>
+  </si>
+  <si>
+    <t>agency_id</t>
+  </si>
+  <si>
+    <t>agency_name</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>coords</t>
+  </si>
+  <si>
+    <t>capacity</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>VBB.zip</t>
+  </si>
+  <si>
+    <t>S-Bahn Berlin GmbH</t>
+  </si>
+  <si>
+    <t>N/A – pure rail operator</t>
+  </si>
+  <si>
+    <t>Oberhavel Verkehrsgesellschaft mbH</t>
+  </si>
+  <si>
+    <t>Oranienburger Depot</t>
+  </si>
+  <si>
+    <t>52.74557505576078, 13.192751192327316</t>
+  </si>
+  <si>
+    <t>Annahofer Str. 1A, 16515 Oranienburg</t>
+  </si>
+  <si>
+    <t>Verkehrsbetriebe Brandenburg an der Havel GmbH</t>
+  </si>
+  <si>
+    <t>Betriebshof Hohenstücken</t>
+  </si>
+  <si>
+    <t>52.428767636612015, 12.533650229827478</t>
+  </si>
+  <si>
+    <t>Upstallstraße 18, 14772 Brandenburg an der Havel</t>
+  </si>
+  <si>
+    <t>Stadtverkehrsgesellschaft mbH Frankfurt (Oder)</t>
+  </si>
+  <si>
+    <t>Betriebshof SVF</t>
+  </si>
+  <si>
+    <t>52.32006508527503, 14.537452913933096</t>
+  </si>
+  <si>
+    <t>Böttnerstraße 1, 15232 Frankfurt (Oder)</t>
+  </si>
+  <si>
+    <t>Havelbus Verkehrsgesellschaft mbH</t>
+  </si>
+  <si>
+    <t>Betriebshof Nauen</t>
+  </si>
+  <si>
+    <t>52.61504442529055, 12.886949093497295</t>
+  </si>
+  <si>
+    <t>Ludwig-Jahn-Straße 1, 14641 Nauen</t>
+  </si>
+  <si>
+    <t>Uckermärkische Verkehrsgesellschaft mbH</t>
+  </si>
+  <si>
+    <t>Uckermärkische Verkehrsgesellschaft</t>
+  </si>
+  <si>
+    <t>53.07084676329792, 14.261990922515063</t>
+  </si>
+  <si>
+    <t>Steinstraße 5, 16303 Schwedt/Oder</t>
+  </si>
+  <si>
+    <t>DB Regio AG</t>
+  </si>
+  <si>
+    <t>Günter Anger Güterverkehrs GmbH &amp; Co. Omnibusvermietung KG</t>
+  </si>
+  <si>
+    <t>Verkehrsbetrieb Potsdam GmbH</t>
+  </si>
+  <si>
+    <t>ViP Betriebshof</t>
+  </si>
+  <si>
+    <t>52.37628875873694, 13.112412796506037</t>
+  </si>
+  <si>
+    <t>Fiktiver Betriebshof Sanssouci</t>
+  </si>
+  <si>
+    <t>52.40497313856915, 13.038360454025698</t>
+  </si>
+  <si>
+    <t>Barnimer Busgesellschaft mbH</t>
+  </si>
+  <si>
+    <t>Betriebshof Nordend</t>
+  </si>
+  <si>
+    <t>52.84967429943032, 13.814701141381143</t>
+  </si>
+  <si>
+    <t>Poratzstraße 68, 16225 Eberswalde</t>
+  </si>
+  <si>
+    <t>Verkehrsgesellschaft Teltow-Fläming mbH</t>
+  </si>
+  <si>
+    <t>Betriebshof Luckenwalde</t>
+  </si>
+  <si>
+    <t>52.08339028518163, 13.160681509418481</t>
+  </si>
+  <si>
+    <t>Forststraße 16, 14943 Luckenwalde</t>
+  </si>
+  <si>
+    <t>Regionale Verkehrsgesellschaft Dahme-Spreewald mbH</t>
+  </si>
+  <si>
+    <t>Nissanstr</t>
+  </si>
+  <si>
+    <t>51.859601652429475, 13.733812378374783</t>
+  </si>
+  <si>
+    <t>Nissanstraße 7, 15926 Luckau</t>
+  </si>
+  <si>
+    <t>Verkehrsmanagement Elbe-Elster GmbH</t>
+  </si>
+  <si>
+    <t>Verkehrsgesellschaft Oberspreewald-Lausitz mbH</t>
+  </si>
+  <si>
+    <t>Fritz Behrendt OHG</t>
+  </si>
+  <si>
+    <t>Glaser</t>
+  </si>
+  <si>
+    <t>Schöneicher Rüdersdorfer Straßenbahn GmbH</t>
+  </si>
+  <si>
+    <t>Strausberger Eisenbahn GmbH</t>
+  </si>
+  <si>
+    <t>Cottbusverkehr GmbH</t>
+  </si>
+  <si>
+    <t>Walther-Rathenau-Straße</t>
+  </si>
+  <si>
+    <t>51.789058228725466, 14.332313340030659</t>
+  </si>
+  <si>
+    <t>Walther-Rathenau-Straße 38, 03044 Cottbus</t>
+  </si>
+  <si>
+    <t>Busverkehr Oder-Spree GmbH</t>
+  </si>
+  <si>
+    <t>James-Watt-Str</t>
+  </si>
+  <si>
+    <t>52.35627786718695, 14.087576948727444</t>
+  </si>
+  <si>
+    <t>James-Watt-Straße 4, 15517 Fürstenwalde</t>
+  </si>
+  <si>
+    <t>NEB Betriebsgesellschaft mbH</t>
+  </si>
+  <si>
+    <t>A. Reich GmbH Busbetrieb</t>
+  </si>
+  <si>
+    <t>Sabinchen Touristik GmbH</t>
+  </si>
+  <si>
+    <t>Busverkehr Gerd Schmidt</t>
+  </si>
+  <si>
+    <t>ORP Ostprignitz-Ruppiner Personennahverkehrsgesellschaft mbH</t>
+  </si>
+  <si>
+    <t>Perleberger Str</t>
+  </si>
+  <si>
+    <t>52.95172629551461, 12.379063105024942</t>
+  </si>
+  <si>
+    <t>Perleberger Str. 64, 16866 Kyritz</t>
+  </si>
+  <si>
+    <t>ODEG Ostdeutsche Eisenbahn GmbH</t>
+  </si>
+  <si>
+    <t>Hanseatische Eisenbahn</t>
+  </si>
+  <si>
+    <t>DB Regio Bus Ost GmbH</t>
+  </si>
+  <si>
+    <t>Lange</t>
+  </si>
+  <si>
+    <t>Berliner Verkehrsbetriebe</t>
+  </si>
+  <si>
+    <t>prignitzbus</t>
+  </si>
+  <si>
+    <t>mobus Märkisch-Oderland Bus GmbH</t>
+  </si>
+  <si>
+    <t>Betriebshof Strausberg</t>
+  </si>
+  <si>
+    <t>52.54829721100754, 13.860390543594225</t>
+  </si>
+  <si>
+    <t>Märkische Straße 3, 15344 Strausberg</t>
+  </si>
+  <si>
+    <t>regiobus Potsdam Mittelmark GmbH</t>
+  </si>
+  <si>
+    <t>Am Betriebshof</t>
+  </si>
+  <si>
+    <t>52.14486495791746, 12.613296403587013</t>
+  </si>
+  <si>
+    <t>Brücker Landstraße 22, 14806 Bad Belzig</t>
+  </si>
+  <si>
+    <t>Mitteldeutsche Regiobahn</t>
+  </si>
+  <si>
+    <t>Betreiber: ecoVista</t>
+  </si>
+  <si>
+    <t>SWU.zip</t>
+  </si>
+  <si>
+    <t>SWU Verkehr GmbH</t>
+  </si>
+  <si>
+    <t>SWU Betriebshof</t>
+  </si>
+  <si>
+    <t>48.39658695394624, 9.967748831666805</t>
+  </si>
+  <si>
+    <t>Bauhoferstraße 9, 89077 Ulm</t>
+  </si>
+  <si>
+    <t>gtfs_DELFI.zip</t>
+  </si>
+  <si>
+    <t>ALV Oberhessen/Marburg/Vogelsberg</t>
+  </si>
+  <si>
+    <t>Betriebshof Fritz Herrmann GmbH</t>
+  </si>
+  <si>
+    <t>50.8210739880651, 8.771314354235805</t>
+  </si>
+  <si>
+    <t>Ernst-Giller-Straße 7 - 35039 Marburg</t>
+  </si>
+  <si>
+    <t>ARGE HRS Omnibus OHG</t>
+  </si>
+  <si>
+    <t>ARGE HRS Betriebshof</t>
+  </si>
+  <si>
+    <t>50.17434484892283, 9.045397135408619</t>
+  </si>
+  <si>
+    <t>Kinzigstraße 10- 63505 Langenselbold</t>
+  </si>
+  <si>
+    <t>ARGE prignitzbus</t>
+  </si>
+  <si>
+    <t>53.10327552712139, 11.482672604389188</t>
+  </si>
+  <si>
+    <t>Lange Felder 3- 19309 Lenzen (Elbe) &amp; Wilsnacker Str. 48 - 19348 Perleberg</t>
+  </si>
+  <si>
+    <t>ASEAG Netliner</t>
+  </si>
+  <si>
+    <t>ASEAG Betriebshof Neuköllner Straße</t>
+  </si>
+  <si>
+    <t>50.78541799579296, 6.129517227474077</t>
+  </si>
+  <si>
+    <t>Neuköllner Straße 1 52068 Aachen</t>
+  </si>
+  <si>
+    <t>vpe.zip</t>
+  </si>
+  <si>
+    <t>kvv-01</t>
+  </si>
+  <si>
+    <t>Albtal-Verkehrs-Gesellschaft mbH</t>
+  </si>
+  <si>
+    <t>Betriebshof und Werkstatt Ettlingen</t>
+  </si>
+  <si>
+    <t>48.93753268361519, 8.411137957421598</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Im Ferning 17-21 76275 Ettlingen </t>
+  </si>
+  <si>
+    <t>AllerBus</t>
+  </si>
+  <si>
+    <t>Eisenbahn- und Omnibusbetrieb</t>
+  </si>
+  <si>
+    <t>52.916429911883746, 9.241323788884339</t>
+  </si>
+  <si>
+    <t>Moorstraße 2a 27283 Verden</t>
+  </si>
+  <si>
+    <t>gesamt_gtfs_MVV.zip</t>
+  </si>
+  <si>
+    <t>mvv-1013</t>
+  </si>
+  <si>
+    <t>AmperBus GmbH</t>
+  </si>
+  <si>
+    <t>Amper Bus Betriebshof</t>
+  </si>
+  <si>
+    <t>48.17835916819891, 11.245401856643896</t>
+  </si>
+  <si>
+    <t>Mühlfeldstraße 8- 82256 Fürstenfeldbruck</t>
+  </si>
+  <si>
+    <t>Andre-Touristk</t>
+  </si>
+  <si>
+    <t>Andre-Touristik Betriebshof</t>
+  </si>
+  <si>
+    <t>50.43881363089824, 6.645480791442084</t>
+  </si>
+  <si>
+    <t>Trierer Str. 1 - 53945 Blankenheim</t>
+  </si>
+  <si>
+    <t>Anklamer Verkehrsgesellschaft</t>
+  </si>
+  <si>
+    <t>Anklamer Betriebshof</t>
+  </si>
+  <si>
+    <t>54.04979879367005, 13.374832325081965</t>
+  </si>
+  <si>
+    <t>Zum Vossberg 7-17498 Weitenhagen</t>
+  </si>
+  <si>
+    <t>Ansbacher Bäder und Verkehrs GmbH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ansbacher Bäder und Verkehrs GmbH Betriebshof </t>
+  </si>
+  <si>
+    <t>49.31072719101067, 10.568297596179125</t>
+  </si>
+  <si>
+    <t>Rügländer Str. 1-91522 Ansbach</t>
+  </si>
+  <si>
+    <t>Arendt Busbetrieb GmbH</t>
+  </si>
+  <si>
+    <t>Arendt Busbetriebshof</t>
+  </si>
+  <si>
+    <t>53.518999037301434, 7.366319272929608</t>
+  </si>
+  <si>
+    <t>Rüskeweg 31-26624 Südbrookmerland</t>
+  </si>
+  <si>
+    <t>Arnold Engelhardt GmbH</t>
+  </si>
+  <si>
+    <t>Engelhardt Betriebshof</t>
+  </si>
+  <si>
+    <t>50.16893693169307, 8.011521326817144</t>
+  </si>
+  <si>
+    <t>Die Haide 15-65321 Heidenrod</t>
+  </si>
+  <si>
+    <t>GTFS_VRS_mit_SPNV.zip</t>
+  </si>
+  <si>
+    <t>BVR Busverkehr Rheinland GmbH</t>
+  </si>
+  <si>
+    <t>Betriebshof Grevenbroich</t>
+  </si>
+  <si>
+    <t>51.081714173790175, 6.628935413701794</t>
+  </si>
+  <si>
+    <t>Marie-Curie-Straße 6-41515 Grevenbroich</t>
+  </si>
+  <si>
+    <t>DL Link</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="7">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -314,41 +490,41 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FF7A4F00"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF7A4F00"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -378,7 +554,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -386,61 +562,32 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-  </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="6">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
+  <cellStyles count="1">
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -499,60 +646,76 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0e2841"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e8e8e8"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="e97132"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196b24"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0f9ed5"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="a02b93"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4ea72e"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
         <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607d"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -584,7 +747,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -608,7 +771,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -668,30 +831,29 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:G38"/>
-  <sheetFormatPr defaultColWidth="10.27734375" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H51"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="50"/>
+    <col min="1" max="2" width="12" customWidth="1"/>
+    <col min="3" max="4" width="50" customWidth="1"/>
+    <col min="5" max="5" width="42" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -714,11 +876,11 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="2">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -730,12 +892,15 @@
       <c r="G2" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="H2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="2">
         <v>32</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -752,11 +917,11 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="2">
         <v>47</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -773,11 +938,11 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="2">
         <v>84</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -794,11 +959,11 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="2">
         <v>92</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -815,11 +980,11 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="2">
         <v>93</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -836,11 +1001,11 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="2">
         <v>108</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -851,11 +1016,11 @@
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="2">
         <v>138</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -866,11 +1031,11 @@
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="2">
         <v>150</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -882,16 +1047,16 @@
       <c r="E10" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="2">
         <v>100</v>
       </c>
       <c r="G10" s="4"/>
     </row>
-    <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="2">
         <v>150</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -903,16 +1068,16 @@
       <c r="E11" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="F11" s="2">
         <v>100</v>
       </c>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="2">
         <v>241</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -929,11 +1094,11 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" s="2">
         <v>246</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -950,11 +1115,11 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" s="2">
         <v>251</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -971,11 +1136,11 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B15" s="2">
         <v>341</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -986,11 +1151,11 @@
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B16" s="2">
         <v>346</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -1001,11 +1166,11 @@
       <c r="F16" s="2"/>
       <c r="G16" s="4"/>
     </row>
-    <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B17" s="2">
         <v>476</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -1016,11 +1181,11 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B18" s="2">
         <v>480</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -1031,11 +1196,11 @@
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B19" s="2">
         <v>486</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -1048,11 +1213,11 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B20" s="2">
         <v>487</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -1065,11 +1230,11 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B21" s="2">
         <v>516</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -1086,11 +1251,11 @@
         <v>58</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B22" s="2">
         <v>566</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -1107,11 +1272,11 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B23" s="2" t="n">
+      <c r="B23" s="2">
         <v>596</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -1124,11 +1289,11 @@
         <v>9</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B24" s="2" t="n">
+      <c r="B24" s="2">
         <v>606</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -1139,11 +1304,11 @@
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
     </row>
-    <row r="25" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B25" s="2" t="n">
+      <c r="B25" s="2">
         <v>706</v>
       </c>
       <c r="C25" s="2" t="s">
@@ -1154,11 +1319,11 @@
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
     </row>
-    <row r="26" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B26" s="2" t="n">
+      <c r="B26" s="2">
         <v>721</v>
       </c>
       <c r="C26" s="2" t="s">
@@ -1169,11 +1334,11 @@
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
     </row>
-    <row r="27" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B27" s="2" t="n">
+      <c r="B27" s="2">
         <v>726</v>
       </c>
       <c r="C27" s="2" t="s">
@@ -1190,11 +1355,11 @@
         <v>70</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B28" s="2">
         <v>731</v>
       </c>
       <c r="C28" s="2" t="s">
@@ -1207,11 +1372,11 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B29" s="2">
         <v>751</v>
       </c>
       <c r="C29" s="2" t="s">
@@ -1224,11 +1389,11 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B30" s="2" t="n">
+      <c r="B30" s="2">
         <v>772</v>
       </c>
       <c r="C30" s="2" t="s">
@@ -1239,11 +1404,11 @@
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
     </row>
-    <row r="31" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B31" s="2" t="n">
+      <c r="B31" s="2">
         <v>781</v>
       </c>
       <c r="C31" s="2" t="s">
@@ -1254,11 +1419,11 @@
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
     </row>
-    <row r="32" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B32" s="2" t="n">
+      <c r="B32" s="2">
         <v>796</v>
       </c>
       <c r="C32" s="2" t="s">
@@ -1269,11 +1434,11 @@
       <c r="F32" s="2"/>
       <c r="G32" s="4"/>
     </row>
-    <row r="33" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="33" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B33" s="2" t="n">
+      <c r="B33" s="2">
         <v>816</v>
       </c>
       <c r="C33" s="2" t="s">
@@ -1284,11 +1449,11 @@
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
     </row>
-    <row r="34" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B34" s="2">
         <v>841</v>
       </c>
       <c r="C34" s="2" t="s">
@@ -1305,11 +1470,11 @@
         <v>80</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="35" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B35" s="2" t="n">
+      <c r="B35" s="2">
         <v>846</v>
       </c>
       <c r="C35" s="2" t="s">
@@ -1326,11 +1491,11 @@
         <v>84</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="36" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B36" s="2" t="n">
+      <c r="B36" s="2">
         <v>856</v>
       </c>
       <c r="C36" s="2" t="s">
@@ -1343,11 +1508,11 @@
         <v>9</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="37" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B37" s="2" t="n">
+      <c r="B37" s="2">
         <v>996</v>
       </c>
       <c r="C37" s="2" t="s">
@@ -1358,11 +1523,11 @@
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
     </row>
-    <row r="38" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="38" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B38" s="2" t="n">
+      <c r="B38" s="2">
         <v>1</v>
       </c>
       <c r="C38" s="2" t="s">
@@ -1379,13 +1544,279 @@
         <v>91</v>
       </c>
     </row>
+    <row r="39" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B39" s="5">
+        <v>8719</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="F39" s="6"/>
+      <c r="G39" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B40" s="5">
+        <v>11981</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="F40" s="6"/>
+      <c r="G40" s="7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B41" s="5">
+        <v>9282</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="F41" s="6"/>
+      <c r="G41" s="7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B42" s="5">
+        <v>11026</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="F42" s="6"/>
+      <c r="G42" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="F43" s="6"/>
+      <c r="G43" s="7" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B44" s="5">
+        <v>12001</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="F44" s="6"/>
+      <c r="G44" s="7" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="F45" s="6"/>
+      <c r="G45" s="7" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B46" s="5">
+        <v>13481</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="F46" s="6"/>
+      <c r="G46" s="7" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B47" s="5">
+        <v>9506</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="F47" s="6"/>
+      <c r="G47" s="7" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B48" s="5">
+        <v>14739</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F48" s="6"/>
+      <c r="G48" s="7" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B49" s="5">
+        <v>14232</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="F49" s="6"/>
+      <c r="G49" s="7" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B50" s="5">
+        <v>8740</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="F50" s="6"/>
+      <c r="G50" s="7" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="B51" s="5">
+        <v>70</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="E51" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="F51" s="6"/>
+      <c r="G51" s="7" t="s">
+        <v>148</v>
+      </c>
+    </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>